<commit_message>
the larp hider (faxom a2 9x19)
</commit_message>
<xml_diff>
--- a/changes/9mm-muzzles.xlsx
+++ b/changes/9mm-muzzles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WhyTh\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC9B5E7-A04B-4AF8-AE67-2BD3875E911D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19190C5E-411E-4704-B538-704B136D233F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>new</t>
   </si>
@@ -225,6 +225,12 @@
   </si>
   <si>
     <t>Kazarov PP-19-01 Vityaz 9x19</t>
+  </si>
+  <si>
+    <t>axom_a2_9x19_flashhider</t>
+  </si>
+  <si>
+    <t>AXOM A2 9x19</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -1192,7 +1198,7 @@
         <v>100</v>
       </c>
       <c r="O4">
-        <f t="shared" ref="O4:O28" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
+        <f t="shared" ref="O4:O29" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
         <v>2.8</v>
       </c>
     </row>
@@ -1387,22 +1393,22 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E10">
         <v>-5</v>
       </c>
       <c r="F10">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -1411,37 +1417,37 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <v>1000</v>
+        <v>150</v>
       </c>
       <c r="O10">
         <f t="shared" si="0"/>
-        <v>6.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="E11">
         <v>-5</v>
       </c>
       <c r="F11">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -1450,7 +1456,7 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <v>-100</v>
+        <v>20</v>
       </c>
       <c r="M11">
         <v>0.04</v>
@@ -1460,288 +1466,288 @@
       </c>
       <c r="O11">
         <f t="shared" si="0"/>
-        <v>2.2999999999999998</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="D12">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="E12">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="F12">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="H12">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>25</v>
+        <v>-100</v>
       </c>
       <c r="M12">
-        <v>-0.05</v>
+        <v>0.04</v>
       </c>
       <c r="N12">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="O12">
-        <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-M12*5</f>
-        <v>7.0750000000000011</v>
+        <f t="shared" si="0"/>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="C13">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="D13">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="E13">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="F13">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="H13">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="I13">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="J13">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M13">
-        <v>-0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="N13">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="O13">
         <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
-        <v>7.9999999999999982</v>
+        <v>7.0750000000000011</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="C14">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="D14">
-        <v>0.22</v>
+        <v>0.23</v>
       </c>
       <c r="E14">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="F14">
         <v>-9</v>
       </c>
       <c r="H14">
+        <v>-0.04</v>
+      </c>
+      <c r="I14">
+        <v>0.12</v>
+      </c>
+      <c r="J14">
+        <v>50</v>
+      </c>
+      <c r="M14">
+        <v>-0.15</v>
+      </c>
+      <c r="N14">
+        <v>1500</v>
+      </c>
+      <c r="O14">
+        <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-M14*5</f>
+        <v>7.9999999999999982</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15">
+        <v>-5</v>
+      </c>
+      <c r="D15">
+        <v>0.22</v>
+      </c>
+      <c r="E15">
+        <v>-7</v>
+      </c>
+      <c r="F15">
+        <v>-9</v>
+      </c>
+      <c r="H15">
         <v>-0.08</v>
       </c>
-      <c r="I14">
+      <c r="I15">
         <v>0.14000000000000001</v>
       </c>
-      <c r="J14">
+      <c r="J15">
         <v>75</v>
       </c>
-      <c r="M14">
+      <c r="M15">
         <v>-0.13</v>
       </c>
-      <c r="N14">
+      <c r="N15">
         <v>1000</v>
       </c>
-      <c r="O14">
+      <c r="O15">
         <f t="shared" si="0"/>
         <v>5.5250000000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>20</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>38</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>-6</v>
       </c>
-      <c r="D15">
+      <c r="D16">
         <v>0.22</v>
       </c>
-      <c r="E15">
+      <c r="E16">
         <v>-7</v>
       </c>
-      <c r="F15">
+      <c r="F16">
         <v>-9</v>
       </c>
-      <c r="H15">
+      <c r="H16">
         <v>-0.08</v>
       </c>
-      <c r="I15">
+      <c r="I16">
         <v>0.14000000000000001</v>
       </c>
-      <c r="J15">
+      <c r="J16">
         <v>75</v>
       </c>
-      <c r="M15">
+      <c r="M16">
         <v>-0.13</v>
       </c>
-      <c r="N15">
+      <c r="N16">
         <v>1000</v>
       </c>
-      <c r="O15">
+      <c r="O16">
         <f t="shared" si="0"/>
         <v>4.5250000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>62</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>63</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>-5</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <v>0.23</v>
       </c>
-      <c r="E16">
+      <c r="E17">
         <v>-10</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <v>-10</v>
       </c>
-      <c r="H16">
+      <c r="H17">
         <v>-0.08</v>
       </c>
-      <c r="I16">
+      <c r="I17">
         <v>0.13</v>
       </c>
-      <c r="J16">
+      <c r="J17">
         <v>25</v>
       </c>
-      <c r="M16">
+      <c r="M17">
         <v>-0.2</v>
       </c>
-      <c r="N16">
+      <c r="N17">
         <v>1200</v>
       </c>
-      <c r="O16">
+      <c r="O17">
         <f t="shared" si="0"/>
         <v>8.2749999999999986</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>31</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>32</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>-5</v>
       </c>
-      <c r="D17">
+      <c r="D18">
         <v>0.24</v>
       </c>
-      <c r="E17">
+      <c r="E18">
         <v>-9</v>
       </c>
-      <c r="F17">
+      <c r="F18">
         <v>-11</v>
       </c>
-      <c r="H17">
+      <c r="H18">
         <v>-0.05</v>
       </c>
-      <c r="I17">
+      <c r="I18">
         <v>0.14000000000000001</v>
       </c>
-      <c r="J17">
+      <c r="J18">
         <v>100</v>
       </c>
-      <c r="M17">
+      <c r="M18">
         <v>-0.18</v>
       </c>
-      <c r="N17">
+      <c r="N18">
         <v>1000</v>
       </c>
-      <c r="O17">
+      <c r="O18">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18">
-        <v>-6</v>
-      </c>
-      <c r="D18">
-        <v>0.19</v>
-      </c>
-      <c r="E18">
-        <v>-8</v>
-      </c>
-      <c r="F18">
-        <v>-12</v>
-      </c>
-      <c r="H18">
-        <v>-0.06</v>
-      </c>
-      <c r="I18">
-        <v>0.15</v>
-      </c>
-      <c r="J18">
-        <v>75</v>
-      </c>
-      <c r="M18">
-        <v>-0.1</v>
-      </c>
-      <c r="N18">
-        <v>1500</v>
-      </c>
-      <c r="O18">
-        <f t="shared" si="0"/>
-        <v>7.5249999999999986</v>
-      </c>
-    </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C19">
         <v>-6</v>
@@ -1777,82 +1783,85 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="B20" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="C20">
+        <v>-6</v>
+      </c>
+      <c r="D20">
+        <v>0.19</v>
+      </c>
+      <c r="E20">
         <v>-8</v>
       </c>
-      <c r="D20">
-        <v>0.25</v>
-      </c>
-      <c r="E20">
-        <v>-6</v>
-      </c>
       <c r="F20">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="H20">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="I20">
-        <v>0.14000000000000001</v>
+        <v>0.15</v>
       </c>
       <c r="J20">
-        <v>200</v>
+        <v>75</v>
+      </c>
+      <c r="M20">
+        <v>-0.1</v>
       </c>
       <c r="N20">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="O20">
         <f t="shared" si="0"/>
-        <v>4.1000000000000014</v>
+        <v>7.5249999999999986</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="D21">
-        <v>0.03</v>
+        <v>0.25</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>-14</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>-0.08</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J21">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="N21">
-        <v>300</v>
+        <v>2000</v>
       </c>
       <c r="O21">
         <f t="shared" si="0"/>
-        <v>-0.6</v>
+        <v>4.1000000000000014</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1883,140 +1892,176 @@
         <v>-0.6</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0.03</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>300</v>
+      </c>
+      <c r="O23">
+        <f t="shared" si="0"/>
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>47</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="C24">
+      <c r="C25">
         <v>-4</v>
       </c>
-      <c r="D24">
+      <c r="D25">
         <v>0.09</v>
       </c>
-      <c r="E24">
+      <c r="E25">
         <v>-9</v>
       </c>
-      <c r="F24">
+      <c r="F25">
         <v>-8</v>
       </c>
-      <c r="H24">
+      <c r="H25">
         <v>-0.03</v>
       </c>
-      <c r="I24">
+      <c r="I25">
         <v>0.09</v>
       </c>
-      <c r="J24">
+      <c r="J25">
         <v>35</v>
       </c>
-      <c r="M24">
+      <c r="M25">
         <v>-0.08</v>
       </c>
-      <c r="N24">
+      <c r="N25">
         <v>1500</v>
       </c>
-      <c r="O24">
+      <c r="O25">
         <f t="shared" si="0"/>
         <v>8.4250000000000007</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>49</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>50</v>
       </c>
-      <c r="C25">
+      <c r="C26">
         <v>-3</v>
       </c>
-      <c r="D25">
+      <c r="D26">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E25">
+      <c r="E26">
         <v>-3</v>
       </c>
-      <c r="F25">
+      <c r="F26">
         <v>-2</v>
       </c>
-      <c r="H25">
+      <c r="H26">
         <v>-0.02</v>
       </c>
-      <c r="I25">
+      <c r="I26">
         <v>0.05</v>
       </c>
-      <c r="J25">
+      <c r="J26">
         <v>25</v>
       </c>
-      <c r="M25">
+      <c r="M26">
         <v>-0.04</v>
       </c>
-      <c r="N25">
+      <c r="N26">
         <v>1000</v>
       </c>
-      <c r="O25">
+      <c r="O26">
         <f t="shared" si="0"/>
         <v>0.47499999999999992</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>51</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>52</v>
       </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
         <v>0.02</v>
       </c>
-      <c r="N26">
-        <v>0</v>
-      </c>
-      <c r="O26">
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
         <f t="shared" si="0"/>
         <v>-0.4</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>30</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>35</v>
       </c>
-      <c r="C28">
+      <c r="C29">
         <v>-5</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <v>0.26</v>
       </c>
-      <c r="E28">
+      <c r="E29">
         <v>-12</v>
       </c>
-      <c r="F28">
+      <c r="F29">
         <v>-16</v>
       </c>
-      <c r="H28">
+      <c r="H29">
         <v>-0.1</v>
       </c>
-      <c r="I28">
+      <c r="I29">
         <v>0.15</v>
       </c>
-      <c r="J28">
+      <c r="J29">
         <v>-180</v>
       </c>
-      <c r="M28">
+      <c r="M29">
         <v>-0.25</v>
       </c>
-      <c r="N28">
+      <c r="N29">
         <v>3000</v>
       </c>
-      <c r="O28">
+      <c r="O29">
         <f t="shared" si="0"/>
         <v>12.600000000000001</v>
       </c>

</xml_diff>

<commit_message>
add egs orthocone to 9mm muzzle sheet
</commit_message>
<xml_diff>
--- a/changes/9mm-muzzles.xlsx
+++ b/changes/9mm-muzzles.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>new</t>
   </si>
@@ -231,6 +231,18 @@
   </si>
   <si>
     <t>AXOM A2 9x19</t>
+  </si>
+  <si>
+    <t>egs_orthocone_45_9x19_piston</t>
+  </si>
+  <si>
+    <t>EGS Orthocone 45 9x19 Piston</t>
+  </si>
+  <si>
+    <t>egs_orthocone_suppressor</t>
+  </si>
+  <si>
+    <t>EGS Orthocone Suppressor</t>
   </si>
 </sst>
 </file>
@@ -1071,7 +1083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -2066,6 +2078,72 @@
         <v>12.600000000000001</v>
       </c>
     </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0.03</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="N31">
+        <v>400</v>
+      </c>
+      <c r="O31">
+        <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-M31*5</f>
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32">
+        <v>-5</v>
+      </c>
+      <c r="D32">
+        <v>0.14</v>
+      </c>
+      <c r="E32">
+        <v>-10</v>
+      </c>
+      <c r="F32">
+        <v>-10</v>
+      </c>
+      <c r="H32">
+        <v>-0.07</v>
+      </c>
+      <c r="I32">
+        <v>0.1</v>
+      </c>
+      <c r="J32">
+        <v>75</v>
+      </c>
+      <c r="M32">
+        <v>-0.15</v>
+      </c>
+      <c r="N32">
+        <v>2600</v>
+      </c>
+      <c r="O32">
+        <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-M32*5</f>
+        <v>9.525</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update 9mm-muzzles, move p226 comp
</commit_message>
<xml_diff>
--- a/changes/9mm-muzzles.xlsx
+++ b/changes/9mm-muzzles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WhyTh\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19190C5E-411E-4704-B538-704B136D233F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C64365C-61EC-4268-AA9C-78F1918C202E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>new</t>
   </si>
@@ -122,9 +122,6 @@
     <t>Wasatch Arms Comp Weight 10mm Compensator for Glock 20</t>
   </si>
   <si>
-    <t>Radian Weapons Glock 17 Gen5 AFTERBURNER Micro Compensator</t>
-  </si>
-  <si>
     <t>hk_mp5sd_9x19_suppressor</t>
   </si>
   <si>
@@ -194,9 +191,6 @@
     <t>Resiliant Suppressors Obsidian9 9x19 Cap</t>
   </si>
   <si>
-    <t>ardian_weapons_glock17_afterburner_micro_compensator</t>
-  </si>
-  <si>
     <t>IPS 1" 9x19</t>
   </si>
   <si>
@@ -243,6 +237,36 @@
   </si>
   <si>
     <t>EGS Orthocone Suppressor</t>
+  </si>
+  <si>
+    <t>suppressors_inc_9x19_thread_protector</t>
+  </si>
+  <si>
+    <t>Suppressors Inc. 9x19</t>
+  </si>
+  <si>
+    <t>sic_sturmer_p_series_9x19_thread_protector</t>
+  </si>
+  <si>
+    <t>Sic Stürmer P-Series 9x19</t>
+  </si>
+  <si>
+    <t>vai_9x19_thread_protector</t>
+  </si>
+  <si>
+    <t>VAI 9x19</t>
+  </si>
+  <si>
+    <t>everetts_sic_226_229_duty_compensator</t>
+  </si>
+  <si>
+    <t>Everetts Machining SIC 226/229 Duty</t>
+  </si>
+  <si>
+    <t>ardian_kosch_catalyst_micro_compensator</t>
+  </si>
+  <si>
+    <t>Ardian KOSCH Catalyst Micro</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
@@ -1118,7 +1142,7 @@
         <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
         <v>9</v>
@@ -1133,7 +1157,7 @@
         <v>12</v>
       </c>
       <c r="M2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N2" t="s">
         <v>13</v>
@@ -1144,10 +1168,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -1210,64 +1234,64 @@
         <v>100</v>
       </c>
       <c r="O4">
-        <f t="shared" ref="O4:O29" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
+        <f t="shared" ref="O4:O33" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
         <v>2.8</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="C5">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
       </c>
       <c r="J5">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N5">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
-        <v>-3.4500000000000006</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="C6">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="D6">
-        <v>7.0000000000000007E-2</v>
+        <v>0.01</v>
       </c>
       <c r="E6">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1276,34 +1300,34 @@
         <v>0</v>
       </c>
       <c r="J6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
-        <v>5.85</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="C7">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="E7">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1312,76 +1336,70 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>20</v>
-      </c>
-      <c r="M7">
-        <v>7.0000000000000007E-2</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
-        <v>7.55</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C8">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="D8">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="E8">
-        <v>-7</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>-9</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="I8">
         <v>0</v>
       </c>
       <c r="J8">
-        <v>20</v>
-      </c>
-      <c r="M8">
-        <v>0.04</v>
+        <v>30</v>
       </c>
       <c r="N8">
-        <v>1800</v>
+        <v>500</v>
       </c>
       <c r="O8">
         <f t="shared" si="0"/>
-        <v>7.8999999999999995</v>
+        <v>-3.4500000000000006</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="C9">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="D9">
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E9">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="F9">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1390,34 +1408,31 @@
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0.03</v>
+        <v>10</v>
       </c>
       <c r="N9">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="O9">
         <f t="shared" si="0"/>
-        <v>7.0500000000000007</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D10">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E10">
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="F10">
         <v>-6</v>
@@ -1429,37 +1444,37 @@
         <v>0</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N10">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="O10">
         <f t="shared" si="0"/>
-        <v>7.6</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="D11">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E11">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="F11">
-        <v>-5</v>
+        <v>-9</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -1474,28 +1489,28 @@
         <v>0.04</v>
       </c>
       <c r="N11">
-        <v>1000</v>
+        <v>1800</v>
       </c>
       <c r="O11">
         <f t="shared" si="0"/>
-        <v>6.1</v>
+        <v>7.8999999999999995</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="C12">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="D12">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="E12">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="F12">
         <v>-7</v>
@@ -1507,109 +1522,109 @@
         <v>0</v>
       </c>
       <c r="J12">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="M12">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="N12">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="O12">
         <f t="shared" si="0"/>
-        <v>2.2999999999999998</v>
+        <v>7.0500000000000007</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="C13">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D13">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="E13">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="F13">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="H13">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="M13">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="N13">
-        <v>900</v>
+        <v>150</v>
       </c>
       <c r="O13">
-        <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
-        <v>7.0750000000000011</v>
+        <f t="shared" si="0"/>
+        <v>7.6</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="C14">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>0.23</v>
+        <v>0.04</v>
       </c>
       <c r="E14">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="F14">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="H14">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J14">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="M14">
-        <v>-0.15</v>
+        <v>0.04</v>
       </c>
       <c r="N14">
-        <v>1500</v>
+        <v>500</v>
       </c>
       <c r="O14">
-        <f>C14-D14*20-E14*0.8-F14*0.6-H14*10+I14*15+J14/200-M14*5</f>
-        <v>7.9999999999999982</v>
+        <f t="shared" si="0"/>
+        <v>8.9</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>75</v>
       </c>
       <c r="C15">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="E15">
         <v>-7</v>
@@ -1617,531 +1632,678 @@
       <c r="F15">
         <v>-9</v>
       </c>
-      <c r="H15">
-        <v>-0.08</v>
-      </c>
-      <c r="I15">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="J15">
-        <v>75</v>
-      </c>
       <c r="M15">
-        <v>-0.13</v>
+        <v>0.05</v>
       </c>
       <c r="N15">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="O15">
         <f t="shared" si="0"/>
-        <v>5.5250000000000004</v>
+        <v>8.35</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C16">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="D16">
-        <v>0.22</v>
+        <v>0.11</v>
       </c>
       <c r="E16">
+        <v>-5</v>
+      </c>
+      <c r="F16">
         <v>-7</v>
       </c>
-      <c r="F16">
-        <v>-9</v>
-      </c>
       <c r="H16">
-        <v>-0.08</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>0.14000000000000001</v>
+        <v>0</v>
       </c>
       <c r="J16">
-        <v>75</v>
+        <v>-100</v>
       </c>
       <c r="M16">
-        <v>-0.13</v>
+        <v>0.04</v>
       </c>
       <c r="N16">
         <v>1000</v>
       </c>
       <c r="O16">
         <f t="shared" si="0"/>
-        <v>4.5250000000000004</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="C17">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="D17">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="E17">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="F17">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="H17">
-        <v>-0.08</v>
+        <v>-0.02</v>
       </c>
       <c r="I17">
-        <v>0.13</v>
+        <v>0.06</v>
       </c>
       <c r="J17">
         <v>25</v>
       </c>
       <c r="M17">
-        <v>-0.2</v>
+        <v>-0.05</v>
       </c>
       <c r="N17">
-        <v>1200</v>
+        <v>900</v>
       </c>
       <c r="O17">
-        <f t="shared" si="0"/>
-        <v>8.2749999999999986</v>
+        <f>C17-D17*20-E17*0.8-F17*0.6-H17*10+I17*15+J17/200-M17*5</f>
+        <v>7.0750000000000011</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C18">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="D18">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="E18">
+        <v>-10</v>
+      </c>
+      <c r="F18">
         <v>-9</v>
       </c>
-      <c r="F18">
-        <v>-11</v>
-      </c>
       <c r="H18">
-        <v>-0.05</v>
+        <v>-0.04</v>
       </c>
       <c r="I18">
-        <v>0.14000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="J18">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="M18">
-        <v>-0.18</v>
+        <v>-0.15</v>
       </c>
       <c r="N18">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="O18">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>C18-D18*20-E18*0.8-F18*0.6-H18*10+I18*15+J18/200-M18*5</f>
+        <v>7.9999999999999982</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="C19">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="D19">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="E19">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="F19">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="H19">
-        <v>-0.06</v>
+        <v>-0.08</v>
       </c>
       <c r="I19">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J19">
         <v>75</v>
       </c>
       <c r="M19">
-        <v>-0.1</v>
+        <v>-0.13</v>
       </c>
       <c r="N19">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="O19">
         <f t="shared" si="0"/>
-        <v>7.5249999999999986</v>
+        <v>5.5250000000000004</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C20">
         <v>-6</v>
       </c>
       <c r="D20">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="E20">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="F20">
-        <v>-12</v>
+        <v>-9</v>
       </c>
       <c r="H20">
-        <v>-0.06</v>
+        <v>-0.08</v>
       </c>
       <c r="I20">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J20">
         <v>75</v>
       </c>
       <c r="M20">
-        <v>-0.1</v>
+        <v>-0.13</v>
       </c>
       <c r="N20">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="O20">
         <f t="shared" si="0"/>
-        <v>7.5249999999999986</v>
+        <v>4.5250000000000004</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C21">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="D21">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="E21">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="F21">
-        <v>-14</v>
+        <v>-10</v>
       </c>
       <c r="H21">
         <v>-0.08</v>
       </c>
       <c r="I21">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
       <c r="J21">
-        <v>200</v>
+        <v>25</v>
+      </c>
+      <c r="M21">
+        <v>-0.2</v>
       </c>
       <c r="N21">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="O21">
         <f t="shared" si="0"/>
-        <v>4.1000000000000014</v>
+        <v>8.2749999999999986</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="D22">
-        <v>0.03</v>
+        <v>0.24</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>-9</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J22">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="M22">
+        <v>-0.18</v>
       </c>
       <c r="N22">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="O22">
         <f t="shared" si="0"/>
-        <v>-0.6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="D23">
-        <v>0.03</v>
+        <v>0.19</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>-8</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>-12</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>-0.06</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>75</v>
+      </c>
+      <c r="M23">
+        <v>-0.1</v>
       </c>
       <c r="N23">
-        <v>300</v>
+        <v>1500</v>
       </c>
       <c r="O23">
         <f t="shared" si="0"/>
-        <v>-0.6</v>
+        <v>7.5249999999999986</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24">
+        <v>-6</v>
+      </c>
+      <c r="D24">
+        <v>0.19</v>
+      </c>
+      <c r="E24">
+        <v>-8</v>
+      </c>
+      <c r="F24">
+        <v>-12</v>
+      </c>
+      <c r="H24">
+        <v>-0.06</v>
+      </c>
+      <c r="I24">
+        <v>0.15</v>
+      </c>
+      <c r="J24">
+        <v>75</v>
+      </c>
+      <c r="M24">
+        <v>-0.1</v>
+      </c>
+      <c r="N24">
+        <v>1500</v>
+      </c>
+      <c r="O24">
+        <f t="shared" si="0"/>
+        <v>7.5249999999999986</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="C25">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="D25">
-        <v>0.09</v>
+        <v>0.25</v>
       </c>
       <c r="E25">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="F25">
-        <v>-8</v>
+        <v>-14</v>
       </c>
       <c r="H25">
-        <v>-0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="I25">
-        <v>0.09</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J25">
-        <v>35</v>
-      </c>
-      <c r="M25">
-        <v>-0.08</v>
+        <v>200</v>
       </c>
       <c r="N25">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="O25">
         <f t="shared" si="0"/>
-        <v>8.4250000000000007</v>
+        <v>4.1000000000000014</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C26">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E26">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>-0.02</v>
+        <v>0</v>
       </c>
       <c r="I26">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J26">
-        <v>25</v>
-      </c>
-      <c r="M26">
-        <v>-0.04</v>
+        <v>0</v>
       </c>
       <c r="N26">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="O26">
         <f t="shared" si="0"/>
-        <v>0.47499999999999992</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>0.02</v>
+        <v>0.03</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
       </c>
       <c r="N27">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="O27">
         <f t="shared" si="0"/>
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="B29" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29">
+        <v>-4</v>
+      </c>
+      <c r="D29">
+        <v>0.09</v>
+      </c>
+      <c r="E29">
+        <v>-9</v>
+      </c>
+      <c r="F29">
+        <v>-8</v>
+      </c>
+      <c r="H29">
+        <v>-0.03</v>
+      </c>
+      <c r="I29">
+        <v>0.09</v>
+      </c>
+      <c r="J29">
         <v>35</v>
       </c>
-      <c r="C29">
-        <v>-5</v>
-      </c>
-      <c r="D29">
-        <v>0.26</v>
-      </c>
-      <c r="E29">
-        <v>-12</v>
-      </c>
-      <c r="F29">
-        <v>-16</v>
-      </c>
-      <c r="H29">
-        <v>-0.1</v>
-      </c>
-      <c r="I29">
-        <v>0.15</v>
-      </c>
-      <c r="J29">
-        <v>-180</v>
-      </c>
       <c r="M29">
-        <v>-0.25</v>
+        <v>-0.08</v>
       </c>
       <c r="N29">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="O29">
         <f t="shared" si="0"/>
-        <v>12.600000000000001</v>
+        <v>8.4250000000000007</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30">
+        <v>-3</v>
+      </c>
+      <c r="D30">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E30">
+        <v>-3</v>
+      </c>
+      <c r="F30">
+        <v>-2</v>
+      </c>
+      <c r="H30">
+        <v>-0.02</v>
+      </c>
+      <c r="I30">
+        <v>0.05</v>
+      </c>
+      <c r="J30">
+        <v>25</v>
+      </c>
+      <c r="M30">
+        <v>-0.04</v>
+      </c>
+      <c r="N30">
+        <v>1000</v>
+      </c>
+      <c r="O30">
+        <f t="shared" si="0"/>
+        <v>0.47499999999999992</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>0.02</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <f t="shared" si="0"/>
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33">
+        <v>-5</v>
+      </c>
+      <c r="D33">
+        <v>0.26</v>
+      </c>
+      <c r="E33">
+        <v>-12</v>
+      </c>
+      <c r="F33">
+        <v>-16</v>
+      </c>
+      <c r="H33">
+        <v>-0.1</v>
+      </c>
+      <c r="I33">
+        <v>0.15</v>
+      </c>
+      <c r="J33">
+        <v>-180</v>
+      </c>
+      <c r="M33">
+        <v>-0.25</v>
+      </c>
+      <c r="N33">
+        <v>3000</v>
+      </c>
+      <c r="O33">
+        <f t="shared" si="0"/>
+        <v>12.600000000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0.03</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="N35">
+        <v>400</v>
+      </c>
+      <c r="O35">
+        <f>C35-D35*20-E35*0.8-F35*0.6-H35*10+I35*15+J35/200-M35*5</f>
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>66</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B36" t="s">
         <v>67</v>
       </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
-        <v>0.03</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="N31">
-        <v>400</v>
-      </c>
-      <c r="O31">
-        <f>C31-D31*20-E31*0.8-F31*0.6-H31*10+I31*15+J31/200-M31*5</f>
-        <v>-0.6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>68</v>
-      </c>
-      <c r="B32" t="s">
-        <v>69</v>
-      </c>
-      <c r="C32">
+      <c r="C36">
         <v>-5</v>
       </c>
-      <c r="D32">
-        <v>0.14</v>
-      </c>
-      <c r="E32">
+      <c r="D36">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="E36">
         <v>-10</v>
       </c>
-      <c r="F32">
+      <c r="F36">
         <v>-10</v>
       </c>
-      <c r="H32">
-        <v>-0.07</v>
-      </c>
-      <c r="I32">
+      <c r="H36">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="I36">
         <v>0.1</v>
       </c>
-      <c r="J32">
+      <c r="J36">
         <v>75</v>
       </c>
-      <c r="M32">
+      <c r="M36">
         <v>-0.15</v>
       </c>
-      <c r="N32">
+      <c r="N36">
         <v>2600</v>
       </c>
-      <c r="O32">
-        <f>C32-D32*20-E32*0.8-F32*0.6-H32*10+I32*15+J32/200-M32*5</f>
-        <v>9.525</v>
+      <c r="O36">
+        <f>C36-D36*20-E36*0.8-F36*0.6-H36*10+I36*15+J36/200-M36*5</f>
+        <v>9.5249999999999986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>